<commit_message>
fix #28: show changes to doc link in UI and exported spreadsheet
</commit_message>
<xml_diff>
--- a/resources/xlsx_templates/fond.xlsx
+++ b/resources/xlsx_templates/fond.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jbrandt/code/birddog/resources/xlsx_templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C43F824-193C-A04C-A226-757F4D92DF24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA06C57E-404E-8047-8565-D88D941483F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7940" yWindow="940" windowWidth="38640" windowHeight="19260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="940" windowWidth="36000" windowHeight="19260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Fund {id}" sheetId="3" r:id="rId1"/>
@@ -155,10 +155,10 @@
     <t>{unquoted_url:linked}</t>
   </si>
   <si>
-    <t>xxxxxx</t>
-  </si>
-  <si>
     <t>{edit:nonexistent}</t>
+  </si>
+  <si>
+    <t>{doc_url:doc_link}</t>
   </si>
 </sst>
 </file>
@@ -965,7 +965,7 @@
         <v>12</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C4" s="9"/>
       <c r="D4" s="10"/>
@@ -1252,7 +1252,7 @@
     </row>
     <row r="15" spans="1:28" x14ac:dyDescent="0.2">
       <c r="O15" s="63" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix wiki table parsing, add logging UI, add date to fond template
</commit_message>
<xml_diff>
--- a/resources/xlsx_templates/fond.xlsx
+++ b/resources/xlsx_templates/fond.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jbrandt/code/birddog/resources/xlsx_templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA06C57E-404E-8047-8565-D88D941483F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDC96D4C-4329-EC45-A1DD-8BF4033AA952}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="940" windowWidth="36000" windowHeight="19260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -146,9 +146,6 @@
     <t>reference date:</t>
   </si>
   <si>
-    <t>YYYY-YYYY</t>
-  </si>
-  <si>
     <t>{parent.name}</t>
   </si>
   <si>
@@ -159,6 +156,9 @@
   </si>
   <si>
     <t>{doc_url:doc_link}</t>
+  </si>
+  <si>
+    <t>{dates}</t>
   </si>
 </sst>
 </file>
@@ -852,7 +852,7 @@
   <sheetData>
     <row r="1" spans="1:28" ht="28" x14ac:dyDescent="0.2">
       <c r="A1" s="36" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B1" s="37"/>
       <c r="C1" s="38" t="s">
@@ -926,14 +926,14 @@
     </row>
     <row r="3" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A3" s="47" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="B3" s="12"/>
       <c r="C3" s="5" t="s">
         <v>0</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E3" s="10"/>
       <c r="F3" s="5"/>
@@ -965,7 +965,7 @@
         <v>12</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C4" s="9"/>
       <c r="D4" s="10"/>
@@ -1252,7 +1252,7 @@
     </row>
     <row r="15" spans="1:28" x14ac:dyDescent="0.2">
       <c r="O15" s="63" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
restructure core page logic to be primarily keyed on page title
</commit_message>
<xml_diff>
--- a/resources/xlsx_templates/fond.xlsx
+++ b/resources/xlsx_templates/fond.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jbrandt/code/birddog/resources/xlsx_templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECDE573F-62EF-CF41-B718-7579EA4BF5C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9E3DAD1-153B-4B4D-9EA6-B3C9105991DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="27120" yWindow="12900" windowWidth="36000" windowHeight="19260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -152,9 +152,6 @@
     <t>{dates}</t>
   </si>
   <si>
-    <t>{parent.clean_name}</t>
-  </si>
-  <si>
     <t>=ROWS($A$__FIRST__:$A__LAST__)</t>
   </si>
   <si>
@@ -186,6 +183,9 @@
   </si>
   <si>
     <t>=SUM(F$__FIRST__:F__LAST__)</t>
+  </si>
+  <si>
+    <t>{archive_name}</t>
   </si>
 </sst>
 </file>
@@ -879,7 +879,7 @@
   <sheetData>
     <row r="1" spans="1:28" ht="28" x14ac:dyDescent="0.2">
       <c r="A1" s="36" t="s">
-        <v>39</v>
+        <v>50</v>
       </c>
       <c r="B1" s="37"/>
       <c r="C1" s="38" t="s">
@@ -1029,34 +1029,34 @@
         <v>1</v>
       </c>
       <c r="E5" s="16" t="s">
+        <v>40</v>
+      </c>
+      <c r="F5" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="G5" s="16" t="s">
+        <v>48</v>
+      </c>
+      <c r="H5" s="16" t="s">
+        <v>47</v>
+      </c>
+      <c r="I5" s="17" t="s">
+        <v>46</v>
+      </c>
+      <c r="J5" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="K5" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="L5" s="17" t="s">
+        <v>43</v>
+      </c>
+      <c r="M5" s="18" t="s">
+        <v>42</v>
+      </c>
+      <c r="N5" s="19" t="s">
         <v>41</v>
-      </c>
-      <c r="F5" s="16" t="s">
-        <v>50</v>
-      </c>
-      <c r="G5" s="16" t="s">
-        <v>49</v>
-      </c>
-      <c r="H5" s="16" t="s">
-        <v>48</v>
-      </c>
-      <c r="I5" s="17" t="s">
-        <v>47</v>
-      </c>
-      <c r="J5" s="17" t="s">
-        <v>46</v>
-      </c>
-      <c r="K5" s="17" t="s">
-        <v>45</v>
-      </c>
-      <c r="L5" s="17" t="s">
-        <v>44</v>
-      </c>
-      <c r="M5" s="18" t="s">
-        <v>43</v>
-      </c>
-      <c r="N5" s="19" t="s">
-        <v>42</v>
       </c>
       <c r="O5" s="9"/>
       <c r="P5" s="28"/>
@@ -1225,7 +1225,7 @@
     </row>
     <row r="9" spans="1:28" ht="16" x14ac:dyDescent="0.2">
       <c r="A9" s="27" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B9" s="24" t="s">
         <v>18</v>

</xml_diff>

<commit_message>
fix #50: transliterate fond and opus labels in export headers (finally!)
</commit_message>
<xml_diff>
--- a/resources/xlsx_templates/fond.xlsx
+++ b/resources/xlsx_templates/fond.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10102"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jbrandt/code/birddog/resources/xlsx_templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9E3DAD1-153B-4B4D-9EA6-B3C9105991DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70E45034-7282-4D4D-AA65-7571976C510B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="27120" yWindow="12900" windowWidth="36000" windowHeight="19260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -98,9 +98,6 @@
     <t>{edit:changed}</t>
   </si>
   <si>
-    <t>{id}</t>
-  </si>
-  <si>
     <t>{description}</t>
   </si>
   <si>
@@ -186,6 +183,9 @@
   </si>
   <si>
     <t>{archive_name}</t>
+  </si>
+  <si>
+    <t>{id:transliterated}</t>
   </si>
 </sst>
 </file>
@@ -879,30 +879,30 @@
   <sheetData>
     <row r="1" spans="1:28" ht="28" x14ac:dyDescent="0.2">
       <c r="A1" s="36" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B1" s="37"/>
       <c r="C1" s="38" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D1" s="39"/>
       <c r="E1" s="40"/>
       <c r="F1" s="41"/>
       <c r="G1" s="42" t="s">
-        <v>21</v>
+        <v>50</v>
       </c>
       <c r="H1" s="42"/>
       <c r="I1" s="36"/>
       <c r="J1" s="40"/>
       <c r="K1" s="43" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="L1" s="44"/>
       <c r="M1" s="43" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="N1" s="45" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="O1" s="34"/>
       <c r="P1" s="39"/>
@@ -921,7 +921,7 @@
     </row>
     <row r="2" spans="1:28" ht="19" x14ac:dyDescent="0.2">
       <c r="A2" s="47" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -953,14 +953,14 @@
     </row>
     <row r="3" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A3" s="47" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B3" s="12"/>
       <c r="C3" s="5" t="s">
         <v>0</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E3" s="10"/>
       <c r="F3" s="5"/>
@@ -992,7 +992,7 @@
         <v>12</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C4" s="9"/>
       <c r="D4" s="10"/>
@@ -1029,34 +1029,34 @@
         <v>1</v>
       </c>
       <c r="E5" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="F5" s="16" t="s">
+        <v>48</v>
+      </c>
+      <c r="G5" s="16" t="s">
+        <v>47</v>
+      </c>
+      <c r="H5" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="I5" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="J5" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="K5" s="17" t="s">
+        <v>43</v>
+      </c>
+      <c r="L5" s="17" t="s">
+        <v>42</v>
+      </c>
+      <c r="M5" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="N5" s="19" t="s">
         <v>40</v>
-      </c>
-      <c r="F5" s="16" t="s">
-        <v>49</v>
-      </c>
-      <c r="G5" s="16" t="s">
-        <v>48</v>
-      </c>
-      <c r="H5" s="16" t="s">
-        <v>47</v>
-      </c>
-      <c r="I5" s="17" t="s">
-        <v>46</v>
-      </c>
-      <c r="J5" s="17" t="s">
-        <v>45</v>
-      </c>
-      <c r="K5" s="17" t="s">
-        <v>44</v>
-      </c>
-      <c r="L5" s="17" t="s">
-        <v>43</v>
-      </c>
-      <c r="M5" s="18" t="s">
-        <v>42</v>
-      </c>
-      <c r="N5" s="19" t="s">
-        <v>41</v>
       </c>
       <c r="O5" s="9"/>
       <c r="P5" s="28"/>
@@ -1135,49 +1135,49 @@
     </row>
     <row r="7" spans="1:28" ht="16" x14ac:dyDescent="0.2">
       <c r="A7" s="25" t="s">
+        <v>27</v>
+      </c>
+      <c r="B7" s="56" t="s">
         <v>28</v>
       </c>
-      <c r="B7" s="56" t="s">
+      <c r="C7" s="57" t="s">
         <v>29</v>
       </c>
-      <c r="C7" s="57" t="s">
-        <v>30</v>
-      </c>
       <c r="D7" s="58" t="s">
+        <v>22</v>
+      </c>
+      <c r="E7" s="32" t="s">
+        <v>22</v>
+      </c>
+      <c r="F7" s="32" t="s">
+        <v>22</v>
+      </c>
+      <c r="G7" s="32" t="s">
+        <v>22</v>
+      </c>
+      <c r="H7" s="32" t="s">
+        <v>24</v>
+      </c>
+      <c r="I7" s="32" t="s">
+        <v>22</v>
+      </c>
+      <c r="J7" s="32" t="s">
+        <v>22</v>
+      </c>
+      <c r="K7" s="32" t="s">
+        <v>22</v>
+      </c>
+      <c r="L7" s="32" t="s">
         <v>23</v>
       </c>
-      <c r="E7" s="32" t="s">
-        <v>23</v>
-      </c>
-      <c r="F7" s="32" t="s">
-        <v>23</v>
-      </c>
-      <c r="G7" s="32" t="s">
-        <v>23</v>
-      </c>
-      <c r="H7" s="32" t="s">
-        <v>25</v>
-      </c>
-      <c r="I7" s="32" t="s">
-        <v>23</v>
-      </c>
-      <c r="J7" s="32" t="s">
-        <v>23</v>
-      </c>
-      <c r="K7" s="32" t="s">
-        <v>23</v>
-      </c>
-      <c r="L7" s="32" t="s">
-        <v>24</v>
-      </c>
       <c r="M7" s="59" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="N7" s="59" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="O7" s="33" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="P7" s="13"/>
       <c r="Q7" s="13"/>
@@ -1225,7 +1225,7 @@
     </row>
     <row r="9" spans="1:28" ht="16" x14ac:dyDescent="0.2">
       <c r="A9" s="27" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B9" s="24" t="s">
         <v>18</v>
@@ -1269,17 +1269,17 @@
     </row>
     <row r="13" spans="1:28" x14ac:dyDescent="0.2">
       <c r="O13" s="34" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="14" spans="1:28" x14ac:dyDescent="0.2">
       <c r="O14" s="62" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="15" spans="1:28" x14ac:dyDescent="0.2">
       <c r="O15" s="63" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>